<commit_message>
Update Attendance roster_Splunk Intermediate_08-10 June_VILT29882.xlsx
</commit_message>
<xml_diff>
--- a/Attendance roster_Splunk Intermediate_08-10 June_VILT29882.xlsx
+++ b/Attendance roster_Splunk Intermediate_08-10 June_VILT29882.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\VK_GIT\CISCO_SPLK_IN_08_06_2026\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{369402F6-C408-4737-947C-F1FC4772B0DE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{421B48B9-4341-4F22-9105-66BCF60E43F6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="86" uniqueCount="49">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="86" uniqueCount="50">
   <si>
     <t>Start Date</t>
   </si>
@@ -173,13 +173,16 @@
   </si>
   <si>
     <t>Cloud Lab URL as follows:    https://cloud.cdp.rpsconsulting.in/console/</t>
+  </si>
+  <si>
+    <t>26MMS0140_U11</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="8" x14ac:knownFonts="1">
+  <fonts count="9" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -236,6 +239,13 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <b/>
+      <sz val="10"/>
+      <color rgb="FF000000"/>
+      <name val="Aptos"/>
+      <family val="2"/>
+    </font>
   </fonts>
   <fills count="4">
     <fill>
@@ -553,7 +563,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="35">
+  <cellXfs count="36">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="top"/>
@@ -624,27 +634,28 @@
     <xf numFmtId="15" fontId="1" fillId="2" borderId="21" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="1"/>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="1"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
@@ -936,10 +947,10 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:5" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B1" s="26" t="s">
+      <c r="B1" s="33" t="s">
         <v>7</v>
       </c>
-      <c r="C1" s="27"/>
+      <c r="C1" s="34"/>
       <c r="D1" s="20"/>
     </row>
     <row r="2" spans="1:5" ht="15" thickBot="1" x14ac:dyDescent="0.35"/>
@@ -1208,33 +1219,33 @@
   </cols>
   <sheetData>
     <row r="2" spans="2:5" x14ac:dyDescent="0.3">
-      <c r="B2" s="34" t="s">
+      <c r="B2" s="31" t="s">
         <v>48</v>
       </c>
     </row>
     <row r="4" spans="2:5" x14ac:dyDescent="0.3">
-      <c r="B4" s="28" t="s">
+      <c r="B4" s="26" t="s">
         <v>5</v>
       </c>
-      <c r="C4" s="28" t="s">
+      <c r="C4" s="26" t="s">
         <v>6</v>
       </c>
-      <c r="D4" s="29" t="s">
+      <c r="D4" s="27" t="s">
         <v>46</v>
       </c>
-      <c r="E4" s="29" t="s">
+      <c r="E4" s="27" t="s">
         <v>47</v>
       </c>
     </row>
-    <row r="5" spans="2:5" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="B5" s="30" t="s">
+    <row r="5" spans="2:5" x14ac:dyDescent="0.3">
+      <c r="B5" s="28" t="s">
         <v>8</v>
       </c>
-      <c r="C5" s="30" t="s">
+      <c r="C5" s="28" t="s">
         <v>20</v>
       </c>
-      <c r="D5" s="31" t="s">
-        <v>34</v>
+      <c r="D5" s="35" t="s">
+        <v>49</v>
       </c>
       <c r="E5" s="32" t="s">
         <v>35</v>
@@ -1247,7 +1258,7 @@
       <c r="C6" s="11" t="s">
         <v>21</v>
       </c>
-      <c r="D6" s="31" t="s">
+      <c r="D6" s="29" t="s">
         <v>36</v>
       </c>
       <c r="E6" s="32"/>
@@ -1259,7 +1270,7 @@
       <c r="C7" s="11" t="s">
         <v>22</v>
       </c>
-      <c r="D7" s="31" t="s">
+      <c r="D7" s="29" t="s">
         <v>37</v>
       </c>
       <c r="E7" s="32"/>
@@ -1271,7 +1282,7 @@
       <c r="C8" s="11" t="s">
         <v>23</v>
       </c>
-      <c r="D8" s="31" t="s">
+      <c r="D8" s="29" t="s">
         <v>38</v>
       </c>
       <c r="E8" s="32"/>
@@ -1283,7 +1294,7 @@
       <c r="C9" s="11" t="s">
         <v>24</v>
       </c>
-      <c r="D9" s="31" t="s">
+      <c r="D9" s="29" t="s">
         <v>39</v>
       </c>
       <c r="E9" s="32"/>
@@ -1295,7 +1306,7 @@
       <c r="C10" s="11" t="s">
         <v>25</v>
       </c>
-      <c r="D10" s="31" t="s">
+      <c r="D10" s="29" t="s">
         <v>40</v>
       </c>
       <c r="E10" s="32"/>
@@ -1307,7 +1318,7 @@
       <c r="C11" s="11" t="s">
         <v>26</v>
       </c>
-      <c r="D11" s="31" t="s">
+      <c r="D11" s="29" t="s">
         <v>41</v>
       </c>
       <c r="E11" s="32"/>
@@ -1319,7 +1330,7 @@
       <c r="C12" s="11" t="s">
         <v>27</v>
       </c>
-      <c r="D12" s="31" t="s">
+      <c r="D12" s="29" t="s">
         <v>42</v>
       </c>
       <c r="E12" s="32"/>
@@ -1331,7 +1342,7 @@
       <c r="C13" s="11" t="s">
         <v>28</v>
       </c>
-      <c r="D13" s="31" t="s">
+      <c r="D13" s="29" t="s">
         <v>34</v>
       </c>
       <c r="E13" s="32"/>
@@ -1343,7 +1354,7 @@
       <c r="C14" s="11" t="s">
         <v>29</v>
       </c>
-      <c r="D14" s="31" t="s">
+      <c r="D14" s="29" t="s">
         <v>43</v>
       </c>
       <c r="E14" s="32"/>
@@ -1355,7 +1366,7 @@
       <c r="C15" s="11" t="s">
         <v>30</v>
       </c>
-      <c r="D15" s="31" t="s">
+      <c r="D15" s="29" t="s">
         <v>44</v>
       </c>
       <c r="E15" s="32"/>
@@ -1367,21 +1378,21 @@
       <c r="C16" s="11" t="s">
         <v>31</v>
       </c>
-      <c r="D16" s="31" t="s">
+      <c r="D16" s="29" t="s">
         <v>45</v>
       </c>
       <c r="E16" s="32"/>
     </row>
     <row r="17" spans="2:5" x14ac:dyDescent="0.3">
-      <c r="B17" s="33"/>
-      <c r="C17" s="33"/>
-      <c r="D17" s="33"/>
+      <c r="B17" s="30"/>
+      <c r="C17" s="30"/>
+      <c r="D17" s="30"/>
       <c r="E17" s="32"/>
     </row>
     <row r="18" spans="2:5" x14ac:dyDescent="0.3">
-      <c r="B18" s="33"/>
-      <c r="C18" s="33"/>
-      <c r="D18" s="33"/>
+      <c r="B18" s="30"/>
+      <c r="C18" s="30"/>
+      <c r="D18" s="30"/>
       <c r="E18" s="32"/>
     </row>
   </sheetData>

</xml_diff>